<commit_message>
Working on the next sequencer
</commit_message>
<xml_diff>
--- a/documentation/BeatsAndCkicks.xlsx
+++ b/documentation/BeatsAndCkicks.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guglielmo\repos\the-guitar-dashboard\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gugli\source\guglielmo\the-guitar-dashboard\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{497B5ED9-4609-45CC-95E2-8BDEEFC72AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A8E7E1-17AE-4F7D-AD69-669DC121A5B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="30" windowWidth="38620" windowHeight="21100" xr2:uid="{153345B2-49C5-4FFB-8445-1F4B094FE494}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{153345B2-49C5-4FFB-8445-1F4B094FE494}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="BPM" sheetId="1" r:id="rId1"/>
+    <sheet name="Samples" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>beats per minute</t>
   </si>
@@ -43,10 +44,22 @@
     <t>beat timespan</t>
   </si>
   <si>
-    <t>ckicks per beat</t>
-  </si>
-  <si>
-    <t>ckick timespan (in mS)</t>
+    <t>clicks per beat</t>
+  </si>
+  <si>
+    <t>click timespan (in mS)</t>
+  </si>
+  <si>
+    <t>rample rate</t>
+  </si>
+  <si>
+    <t>samples per block</t>
+  </si>
+  <si>
+    <t>sample timespan (uS)</t>
+  </si>
+  <si>
+    <t>Block timespan (mS)</t>
   </si>
 </sst>
 </file>
@@ -102,9 +115,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -142,7 +155,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -248,7 +261,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -390,7 +403,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -399,12 +412,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{584E9C01-A434-4B21-B6E1-AFE2E5D72704}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="18.62890625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.61328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -412,7 +425,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -421,7 +434,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -429,13 +442,60 @@
         <v>480</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
         <f>B2/B3*1000</f>
         <v>1.0416666666666667</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C63812-8749-42A4-87F7-432CBAA84A13}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="18.61328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <f>1/B1*1000000</f>
+        <v>20.833333333333332</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <f>B2/B1*1000</f>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>